<commit_message>
TTA-16：使用 R-Port 和 P-Port 命名绿表页签 (#16)
* TTA-16：将绿表页签改为接收和发送方向

用 RECEIVE/SEND 替换绿表的 INPUT/OUTPUT 页签名，并保留旧工作簿兼容；同步合并输出命名、样例、测试和用户文档。

Co-authored-by: Copilot <223556219+Copilot@users.noreply.github.com>

* TTA-16：使用 R-Port 和 P-Port 命名绿表页签

将规范页名调整为 R-Port/P-Port，使名称直接对应当前模块端口类型；兼容 RECEIVE/SEND 及 INPUT/OUTPUT，更新合并输出、样例、测试和文档。

Co-authored-by: Copilot <223556219+Copilot@users.noreply.github.com>

* TTA-16：仅兼容旧 INPUT 和 OUTPUT 页签

移除 RECEIVE/SEND 兼容别名，保留新 R-Port/P-Port 页签及旧 INPUT/OUTPUT 工作簿兼容，并同步更新混合页签测试和说明。

Co-authored-by: Copilot <223556219+Copilot@users.noreply.github.com>

---------

Co-authored-by: Tian Yong (uic81119) <uic81119@automotive-wan.com>
Co-authored-by: Copilot <223556219+Copilot@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/test/samples/system/GreenTable/Bcm/LIT.xlsx
+++ b/test/samples/system/GreenTable/Bcm/LIT.xlsx
@@ -6,12 +6,12 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="28680" yWindow="-75" windowWidth="29040" windowHeight="15720" tabRatio="600" firstSheet="0" activeTab="1" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="INPUT" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="OUTPUT" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="R-Port" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="P-Port" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'INPUT'!$A$1:$K$2</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'OUTPUT'!$A$1:$K$2</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'R-Port'!$A$1:$K$2</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'P-Port'!$A$1:$K$2</definedName>
   </definedNames>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
 </workbook>
@@ -620,8 +620,6 @@
           <t>Power mode test</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr"/>
-      <c r="G2" t="inlineStr"/>
       <c r="H2" t="inlineStr">
         <is>
           <t>PowerMode</t>
@@ -780,8 +778,6 @@
           <t>Position lamp test</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr"/>
-      <c r="G2" t="inlineStr"/>
       <c r="H2" t="inlineStr">
         <is>
           <t>PositionActive</t>

</xml_diff>